<commit_message>
Actualiza anclaje t_360 y principalidad a 202606 (desfase 0)
- t_360_cliente: UM=202606, U3M=202606-202604, U6M=202606-202601
- t_nds_principalidad: fch_periodo=2026-06-30
- RCC/inca/maestro_score sin cambios (mantienen sus periodos)
- Diccionario y desfases regenerados acorde

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Hb3U3iwutCWojkc6BQ3F1K
</commit_message>
<xml_diff>
--- a/Diccionario_PEA202606_REP_V2_mod.xlsx
+++ b/Diccionario_PEA202606_REP_V2_mod.xlsx
@@ -785,7 +785,7 @@
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>frecuencia=1; cod_mes=202604</t>
+          <t>frecuencia=1; cod_mes=202606</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
@@ -795,7 +795,7 @@
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>-2 meses</t>
+          <t>0 (anclaje 202606)</t>
         </is>
       </c>
     </row>
@@ -835,7 +835,7 @@
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>cod_mes 202604-202602</t>
+          <t>cod_mes 202606-202604</t>
         </is>
       </c>
       <c r="I7" s="7" t="inlineStr">
@@ -845,7 +845,7 @@
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>-2 a -4 meses</t>
+          <t>0 a -2 meses</t>
         </is>
       </c>
     </row>
@@ -885,7 +885,7 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>cod_mes 202604-202511</t>
+          <t>cod_mes 202606-202601</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
@@ -895,7 +895,7 @@
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>-2 a -7 meses</t>
+          <t>0 a -5 meses</t>
         </is>
       </c>
     </row>
@@ -935,7 +935,7 @@
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>cod_mes=202604</t>
+          <t>cod_mes=202606</t>
         </is>
       </c>
       <c r="I9" s="7" t="inlineStr">
@@ -945,7 +945,7 @@
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
-          <t>-2 meses</t>
+          <t>0 (anclaje 202606)</t>
         </is>
       </c>
     </row>
@@ -985,7 +985,7 @@
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>cod_mes 202604-202602</t>
+          <t>cod_mes 202606-202604</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
@@ -995,7 +995,7 @@
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>-2 a -4 meses</t>
+          <t>0 a -2 meses</t>
         </is>
       </c>
     </row>
@@ -1035,7 +1035,7 @@
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>cod_mes 202604-202511</t>
+          <t>cod_mes 202606-202601</t>
         </is>
       </c>
       <c r="I11" s="7" t="inlineStr">
@@ -1045,7 +1045,7 @@
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
-          <t>-2 a -7 meses</t>
+          <t>0 a -5 meses</t>
         </is>
       </c>
     </row>
@@ -1085,7 +1085,7 @@
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>cod_mes=202604</t>
+          <t>cod_mes=202606</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
@@ -1095,7 +1095,7 @@
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>-2 meses</t>
+          <t>0 (anclaje 202606)</t>
         </is>
       </c>
     </row>
@@ -1135,7 +1135,7 @@
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>cod_mes 202604-202602</t>
+          <t>cod_mes 202606-202604</t>
         </is>
       </c>
       <c r="I13" s="7" t="inlineStr">
@@ -1145,7 +1145,7 @@
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
-          <t>-2 a -4 meses</t>
+          <t>0 a -2 meses</t>
         </is>
       </c>
     </row>
@@ -1185,7 +1185,7 @@
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>cod_mes 202604-202511</t>
+          <t>cod_mes 202606-202601</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
@@ -1195,7 +1195,7 @@
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>-2 a -7 meses</t>
+          <t>0 a -5 meses</t>
         </is>
       </c>
     </row>
@@ -1235,7 +1235,7 @@
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>cod_mes=202604</t>
+          <t>cod_mes=202606</t>
         </is>
       </c>
       <c r="I15" s="7" t="inlineStr">
@@ -1245,7 +1245,7 @@
       </c>
       <c r="J15" s="7" t="inlineStr">
         <is>
-          <t>-2 meses</t>
+          <t>0 (anclaje 202606)</t>
         </is>
       </c>
     </row>
@@ -1285,7 +1285,7 @@
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>cod_mes 202604-202602</t>
+          <t>cod_mes 202606-202604</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>-2 a -4 meses</t>
+          <t>0 a -2 meses</t>
         </is>
       </c>
     </row>
@@ -1335,7 +1335,7 @@
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>cod_mes 202604-202511</t>
+          <t>cod_mes 202606-202601</t>
         </is>
       </c>
       <c r="I17" s="7" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="J17" s="7" t="inlineStr">
         <is>
-          <t>-2 a -7 meses</t>
+          <t>0 a -5 meses</t>
         </is>
       </c>
     </row>
@@ -1385,7 +1385,7 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>cod_mes=202604</t>
+          <t>cod_mes=202606</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1395,7 +1395,7 @@
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>-2 meses</t>
+          <t>0 (anclaje 202606)</t>
         </is>
       </c>
     </row>
@@ -1435,7 +1435,7 @@
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>cod_mes 202604-202602</t>
+          <t>cod_mes 202606-202604</t>
         </is>
       </c>
       <c r="I19" s="7" t="inlineStr">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="J19" s="7" t="inlineStr">
         <is>
-          <t>-2 a -4 meses</t>
+          <t>0 a -2 meses</t>
         </is>
       </c>
     </row>
@@ -1485,7 +1485,7 @@
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>cod_mes 202604-202511</t>
+          <t>cod_mes 202606-202601</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
@@ -1495,7 +1495,7 @@
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>-2 a -7 meses</t>
+          <t>0 a -5 meses</t>
         </is>
       </c>
     </row>
@@ -1535,7 +1535,7 @@
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>cod_mes=202604</t>
+          <t>cod_mes=202606</t>
         </is>
       </c>
       <c r="I21" s="7" t="inlineStr">
@@ -1545,7 +1545,7 @@
       </c>
       <c r="J21" s="7" t="inlineStr">
         <is>
-          <t>-2 meses</t>
+          <t>0 (anclaje 202606)</t>
         </is>
       </c>
     </row>
@@ -1585,7 +1585,7 @@
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>cod_mes 202604-202602</t>
+          <t>cod_mes 202606-202604</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
@@ -1595,7 +1595,7 @@
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>-2 a -4 meses</t>
+          <t>0 a -2 meses</t>
         </is>
       </c>
     </row>
@@ -1635,7 +1635,7 @@
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>cod_mes 202604-202511</t>
+          <t>cod_mes 202606-202601</t>
         </is>
       </c>
       <c r="I23" s="7" t="inlineStr">
@@ -1645,7 +1645,7 @@
       </c>
       <c r="J23" s="7" t="inlineStr">
         <is>
-          <t>-2 a -7 meses</t>
+          <t>0 a -5 meses</t>
         </is>
       </c>
     </row>
@@ -1685,7 +1685,7 @@
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>cod_mes=202604</t>
+          <t>cod_mes=202606</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
@@ -1695,7 +1695,7 @@
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>-2 meses</t>
+          <t>0 (anclaje 202606)</t>
         </is>
       </c>
     </row>
@@ -1735,7 +1735,7 @@
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>cod_mes 202604-202602</t>
+          <t>cod_mes 202606-202604</t>
         </is>
       </c>
       <c r="I25" s="7" t="inlineStr">
@@ -1745,7 +1745,7 @@
       </c>
       <c r="J25" s="7" t="inlineStr">
         <is>
-          <t>-2 a -4 meses</t>
+          <t>0 a -2 meses</t>
         </is>
       </c>
     </row>
@@ -1785,7 +1785,7 @@
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>cod_mes 202604-202511</t>
+          <t>cod_mes 202606-202601</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
@@ -1795,7 +1795,7 @@
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>-2 a -7 meses</t>
+          <t>0 a -5 meses</t>
         </is>
       </c>
     </row>
@@ -1835,7 +1835,7 @@
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>cod_mes 202604-202511</t>
+          <t>cod_mes 202606-202601</t>
         </is>
       </c>
       <c r="I27" s="7" t="inlineStr">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="J27" s="7" t="inlineStr">
         <is>
-          <t>-2 a -7 meses</t>
+          <t>0 a -5 meses</t>
         </is>
       </c>
     </row>
@@ -1885,7 +1885,7 @@
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>cod_mes=202604</t>
+          <t>cod_mes=202606</t>
         </is>
       </c>
       <c r="I28" s="4" t="inlineStr">
@@ -1895,7 +1895,7 @@
       </c>
       <c r="J28" s="4" t="inlineStr">
         <is>
-          <t>-2 meses</t>
+          <t>0 (anclaje 202606)</t>
         </is>
       </c>
     </row>
@@ -1935,7 +1935,7 @@
       </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
-          <t>cod_mes 202604-202511</t>
+          <t>cod_mes 202606-202601</t>
         </is>
       </c>
       <c r="I29" s="7" t="inlineStr">
@@ -1945,7 +1945,7 @@
       </c>
       <c r="J29" s="7" t="inlineStr">
         <is>
-          <t>-2 a -7 meses</t>
+          <t>0 a -5 meses</t>
         </is>
       </c>
     </row>
@@ -1985,7 +1985,7 @@
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>cod_mes=202604</t>
+          <t>cod_mes=202606</t>
         </is>
       </c>
       <c r="I30" s="4" t="inlineStr">
@@ -1995,7 +1995,7 @@
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>-2 meses</t>
+          <t>0 (anclaje 202606)</t>
         </is>
       </c>
     </row>
@@ -2035,7 +2035,7 @@
       </c>
       <c r="H31" s="7" t="inlineStr">
         <is>
-          <t>cod_mes 202604-202511</t>
+          <t>cod_mes 202606-202601</t>
         </is>
       </c>
       <c r="I31" s="7" t="inlineStr">
@@ -2045,7 +2045,7 @@
       </c>
       <c r="J31" s="7" t="inlineStr">
         <is>
-          <t>-2 a -7 meses</t>
+          <t>0 a -5 meses</t>
         </is>
       </c>
     </row>
@@ -2085,7 +2085,7 @@
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>cod_mes=202604</t>
+          <t>cod_mes=202606</t>
         </is>
       </c>
       <c r="I32" s="4" t="inlineStr">
@@ -2095,7 +2095,7 @@
       </c>
       <c r="J32" s="4" t="inlineStr">
         <is>
-          <t>-2 meses</t>
+          <t>0 (anclaje 202606)</t>
         </is>
       </c>
     </row>
@@ -2135,7 +2135,7 @@
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>cod_mes 202604-202511</t>
+          <t>cod_mes 202606-202601</t>
         </is>
       </c>
       <c r="I33" s="7" t="inlineStr">
@@ -2145,7 +2145,7 @@
       </c>
       <c r="J33" s="7" t="inlineStr">
         <is>
-          <t>-2 a -7 meses</t>
+          <t>0 a -5 meses</t>
         </is>
       </c>
     </row>
@@ -2185,7 +2185,7 @@
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>cod_mes=202604</t>
+          <t>cod_mes=202606</t>
         </is>
       </c>
       <c r="I34" s="4" t="inlineStr">
@@ -2195,7 +2195,7 @@
       </c>
       <c r="J34" s="4" t="inlineStr">
         <is>
-          <t>-2 meses</t>
+          <t>0 (anclaje 202606)</t>
         </is>
       </c>
     </row>
@@ -2235,7 +2235,7 @@
       </c>
       <c r="H35" s="7" t="inlineStr">
         <is>
-          <t>cod_mes 202604-202511</t>
+          <t>cod_mes 202606-202601</t>
         </is>
       </c>
       <c r="I35" s="7" t="inlineStr">
@@ -2245,7 +2245,7 @@
       </c>
       <c r="J35" s="7" t="inlineStr">
         <is>
-          <t>-2 a -7 meses</t>
+          <t>0 a -5 meses</t>
         </is>
       </c>
     </row>
@@ -2285,7 +2285,7 @@
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>cod_mes=202604</t>
+          <t>cod_mes=202606</t>
         </is>
       </c>
       <c r="I36" s="4" t="inlineStr">
@@ -2295,7 +2295,7 @@
       </c>
       <c r="J36" s="4" t="inlineStr">
         <is>
-          <t>-2 meses</t>
+          <t>0 (anclaje 202606)</t>
         </is>
       </c>
     </row>
@@ -2335,7 +2335,7 @@
       </c>
       <c r="H37" s="7" t="inlineStr">
         <is>
-          <t>cod_mes 202604-202511</t>
+          <t>cod_mes 202606-202601</t>
         </is>
       </c>
       <c r="I37" s="7" t="inlineStr">
@@ -2345,7 +2345,7 @@
       </c>
       <c r="J37" s="7" t="inlineStr">
         <is>
-          <t>-2 a -7 meses</t>
+          <t>0 a -5 meses</t>
         </is>
       </c>
     </row>
@@ -2385,7 +2385,7 @@
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>cod_mes=202604</t>
+          <t>cod_mes=202606</t>
         </is>
       </c>
       <c r="I38" s="4" t="inlineStr">
@@ -2395,7 +2395,7 @@
       </c>
       <c r="J38" s="4" t="inlineStr">
         <is>
-          <t>-2 meses</t>
+          <t>0 (anclaje 202606)</t>
         </is>
       </c>
     </row>
@@ -2435,7 +2435,7 @@
       </c>
       <c r="H39" s="7" t="inlineStr">
         <is>
-          <t>cod_mes 202604-202511</t>
+          <t>cod_mes 202606-202601</t>
         </is>
       </c>
       <c r="I39" s="7" t="inlineStr">
@@ -2445,7 +2445,7 @@
       </c>
       <c r="J39" s="7" t="inlineStr">
         <is>
-          <t>-2 a -7 meses</t>
+          <t>0 a -5 meses</t>
         </is>
       </c>
     </row>
@@ -2485,7 +2485,7 @@
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>cod_mes=202604</t>
+          <t>cod_mes=202606</t>
         </is>
       </c>
       <c r="I40" s="4" t="inlineStr">
@@ -2495,7 +2495,7 @@
       </c>
       <c r="J40" s="4" t="inlineStr">
         <is>
-          <t>-2 meses</t>
+          <t>0 (anclaje 202606)</t>
         </is>
       </c>
     </row>
@@ -2535,7 +2535,7 @@
       </c>
       <c r="H41" s="7" t="inlineStr">
         <is>
-          <t>cod_mes 202604-202511</t>
+          <t>cod_mes 202606-202601</t>
         </is>
       </c>
       <c r="I41" s="7" t="inlineStr">
@@ -2545,7 +2545,7 @@
       </c>
       <c r="J41" s="7" t="inlineStr">
         <is>
-          <t>-2 a -7 meses</t>
+          <t>0 a -5 meses</t>
         </is>
       </c>
     </row>
@@ -2585,7 +2585,7 @@
       </c>
       <c r="H42" s="4" t="inlineStr">
         <is>
-          <t>cod_mes=202604</t>
+          <t>cod_mes=202606</t>
         </is>
       </c>
       <c r="I42" s="4" t="inlineStr">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="J42" s="4" t="inlineStr">
         <is>
-          <t>-2 meses</t>
+          <t>0 (anclaje 202606)</t>
         </is>
       </c>
     </row>
@@ -2635,7 +2635,7 @@
       </c>
       <c r="H43" s="7" t="inlineStr">
         <is>
-          <t>cod_mes 202604-202511</t>
+          <t>cod_mes 202606-202601</t>
         </is>
       </c>
       <c r="I43" s="7" t="inlineStr">
@@ -2645,7 +2645,7 @@
       </c>
       <c r="J43" s="7" t="inlineStr">
         <is>
-          <t>-2 a -7 meses</t>
+          <t>0 a -5 meses</t>
         </is>
       </c>
     </row>
@@ -2685,7 +2685,7 @@
       </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
-          <t>cod_mes=202604</t>
+          <t>cod_mes=202606</t>
         </is>
       </c>
       <c r="I44" s="4" t="inlineStr">
@@ -2695,7 +2695,7 @@
       </c>
       <c r="J44" s="4" t="inlineStr">
         <is>
-          <t>-2 meses</t>
+          <t>0 (anclaje 202606)</t>
         </is>
       </c>
     </row>
@@ -2735,7 +2735,7 @@
       </c>
       <c r="H45" s="7" t="inlineStr">
         <is>
-          <t>cod_mes 202604-202511</t>
+          <t>cod_mes 202606-202601</t>
         </is>
       </c>
       <c r="I45" s="7" t="inlineStr">
@@ -2745,7 +2745,7 @@
       </c>
       <c r="J45" s="7" t="inlineStr">
         <is>
-          <t>-2 a -7 meses</t>
+          <t>0 a -5 meses</t>
         </is>
       </c>
     </row>
@@ -2785,7 +2785,7 @@
       </c>
       <c r="H46" s="4" t="inlineStr">
         <is>
-          <t>cod_mes=202604</t>
+          <t>cod_mes=202606</t>
         </is>
       </c>
       <c r="I46" s="4" t="inlineStr">
@@ -2795,7 +2795,7 @@
       </c>
       <c r="J46" s="4" t="inlineStr">
         <is>
-          <t>-2 meses</t>
+          <t>0 (anclaje 202606)</t>
         </is>
       </c>
     </row>
@@ -2835,7 +2835,7 @@
       </c>
       <c r="H47" s="7" t="inlineStr">
         <is>
-          <t>cod_mes 202604-202511</t>
+          <t>cod_mes 202606-202601</t>
         </is>
       </c>
       <c r="I47" s="7" t="inlineStr">
@@ -2845,7 +2845,7 @@
       </c>
       <c r="J47" s="7" t="inlineStr">
         <is>
-          <t>-2 a -7 meses</t>
+          <t>0 a -5 meses</t>
         </is>
       </c>
     </row>
@@ -2895,7 +2895,7 @@
       </c>
       <c r="J48" s="4" t="inlineStr">
         <is>
-          <t>-2 a -4 meses</t>
+          <t>0 a -2 meses</t>
         </is>
       </c>
     </row>
@@ -2945,7 +2945,7 @@
       </c>
       <c r="J49" s="7" t="inlineStr">
         <is>
-          <t>-2 a -4 meses</t>
+          <t>0 a -2 meses</t>
         </is>
       </c>
     </row>
@@ -2995,7 +2995,7 @@
       </c>
       <c r="J50" s="4" t="inlineStr">
         <is>
-          <t>-2 a -4 meses</t>
+          <t>0 a -2 meses</t>
         </is>
       </c>
     </row>
@@ -3045,7 +3045,7 @@
       </c>
       <c r="J51" s="7" t="inlineStr">
         <is>
-          <t>-2 a -4 meses</t>
+          <t>0 a -2 meses</t>
         </is>
       </c>
     </row>
@@ -3095,7 +3095,7 @@
       </c>
       <c r="J52" s="4" t="inlineStr">
         <is>
-          <t>-2 a -7 meses</t>
+          <t>0 a -5 meses</t>
         </is>
       </c>
     </row>
@@ -3145,7 +3145,7 @@
       </c>
       <c r="J53" s="7" t="inlineStr">
         <is>
-          <t>-2 a -7 meses</t>
+          <t>0 a -5 meses</t>
         </is>
       </c>
     </row>
@@ -3185,7 +3185,7 @@
       </c>
       <c r="H54" s="4" t="inlineStr">
         <is>
-          <t>fch_periodo=2026-04-30</t>
+          <t>fch_periodo=2026-06-30</t>
         </is>
       </c>
       <c r="I54" s="4" t="inlineStr">
@@ -3195,7 +3195,7 @@
       </c>
       <c r="J54" s="4" t="inlineStr">
         <is>
-          <t>-2 meses</t>
+          <t>0 (anclaje 202606)</t>
         </is>
       </c>
     </row>
@@ -3715,12 +3715,12 @@
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>frecuencia=1; cod_mes 202604-202511</t>
+          <t>frecuencia=1; cod_mes 202606-202601</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>-2 a -7</t>
+          <t>0 a -5</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -3752,12 +3752,12 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>fch_periodo=2026-04-30</t>
+          <t>fch_periodo=2026-06-30</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>-2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -3927,7 +3927,7 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>ultimo mes = 202604</t>
+          <t>ultimo mes = 202606</t>
         </is>
       </c>
     </row>
@@ -3939,7 +3939,7 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>202604, 202603, 202602 (promedio)</t>
+          <t>202606, 202605, 202604 (promedio)</t>
         </is>
       </c>
     </row>
@@ -3951,7 +3951,7 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>202604, 202603, 202602, 202601, 202512, 202511</t>
+          <t>202606, 202605, 202604, 202603, 202602, 202601</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reconstruye query desde version real e integra variables nuevas
- Parte del query original del usuario (edad_num, rk_ing_num,
  rcc_castigo_num, pasivo_num) y agrega encima: saldos t_360
  txs/planilla/tc UM/U3M/U6M (anclaje 202606), flags 0/1/null,
  ratios, entidades castigo vida, principalidad, sexo/estado_civil,
  nivel_profesional/tipinstitucion.
- Diccionario ampliado a 70 variables con base de origen y desfase.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Hb3U3iwutCWojkc6BQ3F1K
</commit_message>
<xml_diff>
--- a/Diccionario_PEA202606_REP_V2_mod.xlsx
+++ b/Diccionario_PEA202606_REP_V2_mod.xlsx
@@ -482,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J56"/>
+  <dimension ref="A1:J71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3296,6 +3296,756 @@
       <c r="J56" s="4" t="inlineStr">
         <is>
           <t>corte -3 / ventana 24M</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>edad_num</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>Edad del cliente (valor numerico)</t>
+        </is>
+      </c>
+      <c r="D57" s="7" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="E57" s="7" t="inlineStr">
+        <is>
+          <t>ds_rtd_rskvol_indicadores_pea</t>
+        </is>
+      </c>
+      <c r="F57" s="7" t="inlineStr">
+        <is>
+          <t>e_perm_aws</t>
+        </is>
+      </c>
+      <c r="G57" s="7" t="inlineStr">
+        <is>
+          <t>p_fecinformacion (poblacion PEA)</t>
+        </is>
+      </c>
+      <c r="H57" s="7" t="inlineStr">
+        <is>
+          <t>p_fecinformacion=20260616</t>
+        </is>
+      </c>
+      <c r="I57" s="7" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="J57" s="7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>rk_ing_num</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>Renta / ingreso (valor numerico)</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="inlineStr">
+        <is>
+          <t>ds_rtd_rskvol_indicadores_pea</t>
+        </is>
+      </c>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>e_perm_aws</t>
+        </is>
+      </c>
+      <c r="G58" s="4" t="inlineStr">
+        <is>
+          <t>p_fecinformacion (poblacion PEA)</t>
+        </is>
+      </c>
+      <c r="H58" s="4" t="inlineStr">
+        <is>
+          <t>p_fecinformacion=20260616</t>
+        </is>
+      </c>
+      <c r="I58" s="4" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="J58" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>monto_castigado_total</t>
+        </is>
+      </c>
+      <c r="C59" s="7" t="inlineStr">
+        <is>
+          <t>Saldo castigado total (cuentas 8113/8123/8133)</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="inlineStr">
+        <is>
+          <t>t_fact_report_rcc_rsk</t>
+        </is>
+      </c>
+      <c r="F59" s="7" t="inlineStr">
+        <is>
+          <t>e_perm_aws</t>
+        </is>
+      </c>
+      <c r="G59" s="7" t="inlineStr">
+        <is>
+          <t>key_value + tip_doc</t>
+        </is>
+      </c>
+      <c r="H59" s="7" t="inlineStr">
+        <is>
+          <t>codmes=202604 (ventana 24m)</t>
+        </is>
+      </c>
+      <c r="I59" s="7" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="J59" s="7" t="inlineStr">
+        <is>
+          <t>-2 meses</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>monto_castigado_ibk</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>Saldo castigado IBK (00002)</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="inlineStr">
+        <is>
+          <t>t_fact_report_rcc_rsk</t>
+        </is>
+      </c>
+      <c r="F60" s="4" t="inlineStr">
+        <is>
+          <t>e_perm_aws</t>
+        </is>
+      </c>
+      <c r="G60" s="4" t="inlineStr">
+        <is>
+          <t>key_value + tip_doc</t>
+        </is>
+      </c>
+      <c r="H60" s="4" t="inlineStr">
+        <is>
+          <t>codmes=202604</t>
+        </is>
+      </c>
+      <c r="I60" s="4" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="J60" s="4" t="inlineStr">
+        <is>
+          <t>-2 meses</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>monto_castigado_otros</t>
+        </is>
+      </c>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>Saldo castigado otras entidades (&lt;&gt;00002)</t>
+        </is>
+      </c>
+      <c r="D61" s="7" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="inlineStr">
+        <is>
+          <t>t_fact_report_rcc_rsk</t>
+        </is>
+      </c>
+      <c r="F61" s="7" t="inlineStr">
+        <is>
+          <t>e_perm_aws</t>
+        </is>
+      </c>
+      <c r="G61" s="7" t="inlineStr">
+        <is>
+          <t>key_value + tip_doc</t>
+        </is>
+      </c>
+      <c r="H61" s="7" t="inlineStr">
+        <is>
+          <t>codmes=202604</t>
+        </is>
+      </c>
+      <c r="I61" s="7" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="J61" s="7" t="inlineStr">
+        <is>
+          <t>-2 meses</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>nro_entidades_castigo</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>Nro entidades distintas con castigo (actual)</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>bigint</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="inlineStr">
+        <is>
+          <t>t_fact_report_rcc_rsk</t>
+        </is>
+      </c>
+      <c r="F62" s="4" t="inlineStr">
+        <is>
+          <t>e_perm_aws</t>
+        </is>
+      </c>
+      <c r="G62" s="4" t="inlineStr">
+        <is>
+          <t>key_value + tip_doc</t>
+        </is>
+      </c>
+      <c r="H62" s="4" t="inlineStr">
+        <is>
+          <t>codmes=202604</t>
+        </is>
+      </c>
+      <c r="I62" s="4" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="J62" s="4" t="inlineStr">
+        <is>
+          <t>-2 meses</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>max_dias_mora_castigo</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>Maximo dias de mora del castigo</t>
+        </is>
+      </c>
+      <c r="D63" s="7" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="inlineStr">
+        <is>
+          <t>t_fact_report_rcc_rsk</t>
+        </is>
+      </c>
+      <c r="F63" s="7" t="inlineStr">
+        <is>
+          <t>e_perm_aws</t>
+        </is>
+      </c>
+      <c r="G63" s="7" t="inlineStr">
+        <is>
+          <t>key_value + tip_doc</t>
+        </is>
+      </c>
+      <c r="H63" s="7" t="inlineStr">
+        <is>
+          <t>codmes=202604</t>
+        </is>
+      </c>
+      <c r="I63" s="7" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="J63" s="7" t="inlineStr">
+        <is>
+          <t>-2 meses</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>meses_desde_ultimo_castigo</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>Meses desde el ultimo reporte de castigo</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="inlineStr">
+        <is>
+          <t>t_fact_report_rcc_rsk</t>
+        </is>
+      </c>
+      <c r="F64" s="4" t="inlineStr">
+        <is>
+          <t>e_perm_aws</t>
+        </is>
+      </c>
+      <c r="G64" s="4" t="inlineStr">
+        <is>
+          <t>key_value + tip_doc</t>
+        </is>
+      </c>
+      <c r="H64" s="4" t="inlineStr">
+        <is>
+          <t>ventana 24m vs 202604</t>
+        </is>
+      </c>
+      <c r="I64" s="4" t="inlineStr">
+        <is>
+          <t>U24M</t>
+        </is>
+      </c>
+      <c r="J64" s="4" t="inlineStr">
+        <is>
+          <t>-2 meses (ref)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>meses_desde_primer_castigo</t>
+        </is>
+      </c>
+      <c r="C65" s="7" t="inlineStr">
+        <is>
+          <t>Meses desde el primer reporte de castigo</t>
+        </is>
+      </c>
+      <c r="D65" s="7" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="E65" s="7" t="inlineStr">
+        <is>
+          <t>t_fact_report_rcc_rsk</t>
+        </is>
+      </c>
+      <c r="F65" s="7" t="inlineStr">
+        <is>
+          <t>e_perm_aws</t>
+        </is>
+      </c>
+      <c r="G65" s="7" t="inlineStr">
+        <is>
+          <t>key_value + tip_doc</t>
+        </is>
+      </c>
+      <c r="H65" s="7" t="inlineStr">
+        <is>
+          <t>ventana 24m vs 202604</t>
+        </is>
+      </c>
+      <c r="I65" s="7" t="inlineStr">
+        <is>
+          <t>U24M</t>
+        </is>
+      </c>
+      <c r="J65" s="7" t="inlineStr">
+        <is>
+          <t>-2 meses (ref)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>saldo_pasivo_actual</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>Saldo fin de periodo pasivo (mes actual)</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="inlineStr">
+        <is>
+          <t>t_360_cliente</t>
+        </is>
+      </c>
+      <c r="F66" s="4" t="inlineStr">
+        <is>
+          <t>e_perm_aws</t>
+        </is>
+      </c>
+      <c r="G66" s="4" t="inlineStr">
+        <is>
+          <t>cod_tipo_documento + nro_documento</t>
+        </is>
+      </c>
+      <c r="H66" s="4" t="inlineStr">
+        <is>
+          <t>cod_mes=202605</t>
+        </is>
+      </c>
+      <c r="I66" s="4" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="J66" s="4" t="inlineStr">
+        <is>
+          <t>-1 mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" s="6" t="inlineStr">
+        <is>
+          <t>saldo_prom_pasivo</t>
+        </is>
+      </c>
+      <c r="C67" s="7" t="inlineStr">
+        <is>
+          <t>Saldo promedio pasivo (mes actual)</t>
+        </is>
+      </c>
+      <c r="D67" s="7" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="E67" s="7" t="inlineStr">
+        <is>
+          <t>t_360_cliente</t>
+        </is>
+      </c>
+      <c r="F67" s="7" t="inlineStr">
+        <is>
+          <t>e_perm_aws</t>
+        </is>
+      </c>
+      <c r="G67" s="7" t="inlineStr">
+        <is>
+          <t>doc</t>
+        </is>
+      </c>
+      <c r="H67" s="7" t="inlineStr">
+        <is>
+          <t>cod_mes=202605</t>
+        </is>
+      </c>
+      <c r="I67" s="7" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="J67" s="7" t="inlineStr">
+        <is>
+          <t>-1 mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>saldo_activo_actual</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>Saldo fin de periodo activo (mes actual)</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="inlineStr">
+        <is>
+          <t>t_360_cliente</t>
+        </is>
+      </c>
+      <c r="F68" s="4" t="inlineStr">
+        <is>
+          <t>e_perm_aws</t>
+        </is>
+      </c>
+      <c r="G68" s="4" t="inlineStr">
+        <is>
+          <t>doc</t>
+        </is>
+      </c>
+      <c r="H68" s="4" t="inlineStr">
+        <is>
+          <t>cod_mes=202605</t>
+        </is>
+      </c>
+      <c r="I68" s="4" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="J68" s="4" t="inlineStr">
+        <is>
+          <t>-1 mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" s="6" t="inlineStr">
+        <is>
+          <t>prom_saldo_pasivo_u4m</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="inlineStr">
+        <is>
+          <t>Promedio saldo FDP pasivo U4M</t>
+        </is>
+      </c>
+      <c r="D69" s="7" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="E69" s="7" t="inlineStr">
+        <is>
+          <t>t_360_cliente</t>
+        </is>
+      </c>
+      <c r="F69" s="7" t="inlineStr">
+        <is>
+          <t>e_perm_aws</t>
+        </is>
+      </c>
+      <c r="G69" s="7" t="inlineStr">
+        <is>
+          <t>doc</t>
+        </is>
+      </c>
+      <c r="H69" s="7" t="inlineStr">
+        <is>
+          <t>cod_mes 202605-202602</t>
+        </is>
+      </c>
+      <c r="I69" s="7" t="inlineStr">
+        <is>
+          <t>U4M (prom)</t>
+        </is>
+      </c>
+      <c r="J69" s="7" t="inlineStr">
+        <is>
+          <t>-1 a -4 meses</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>max_saldo_pasivo_u6m</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>Maximo saldo FDP pasivo U6M</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="E70" s="4" t="inlineStr">
+        <is>
+          <t>t_360_cliente</t>
+        </is>
+      </c>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
+          <t>e_perm_aws</t>
+        </is>
+      </c>
+      <c r="G70" s="4" t="inlineStr">
+        <is>
+          <t>doc</t>
+        </is>
+      </c>
+      <c r="H70" s="4" t="inlineStr">
+        <is>
+          <t>cod_mes 202605-202512</t>
+        </is>
+      </c>
+      <c r="I70" s="4" t="inlineStr">
+        <is>
+          <t>U6M (max)</t>
+        </is>
+      </c>
+      <c r="J70" s="4" t="inlineStr">
+        <is>
+          <t>-1 a -6 meses</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>nro_meses_con_pasivo_u6m</t>
+        </is>
+      </c>
+      <c r="C71" s="7" t="inlineStr">
+        <is>
+          <t>Nro meses con saldo pasivo&gt;0 en U6M</t>
+        </is>
+      </c>
+      <c r="D71" s="7" t="inlineStr">
+        <is>
+          <t>bigint</t>
+        </is>
+      </c>
+      <c r="E71" s="7" t="inlineStr">
+        <is>
+          <t>t_360_cliente</t>
+        </is>
+      </c>
+      <c r="F71" s="7" t="inlineStr">
+        <is>
+          <t>e_perm_aws</t>
+        </is>
+      </c>
+      <c r="G71" s="7" t="inlineStr">
+        <is>
+          <t>doc</t>
+        </is>
+      </c>
+      <c r="H71" s="7" t="inlineStr">
+        <is>
+          <t>cod_mes 202605-202512</t>
+        </is>
+      </c>
+      <c r="I71" s="7" t="inlineStr">
+        <is>
+          <t>U6M</t>
+        </is>
+      </c>
+      <c r="J71" s="7" t="inlineStr">
+        <is>
+          <t>-1 a -6 meses</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Alinea pasivo_num a anclaje 202606 (desfase 0)
- pasivo_num: cod_mes 202605 -> 202606; U4M=202606-202603; U6M=202606-202601
- RCC castigo se mantiene en 202604 (desfase de disponibilidad RCC)
- Diccionario actualizado: desfases de pasivo a 0

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Hb3U3iwutCWojkc6BQ3F1K
</commit_message>
<xml_diff>
--- a/Diccionario_PEA202606_REP_V2_mod.xlsx
+++ b/Diccionario_PEA202606_REP_V2_mod.xlsx
@@ -3785,7 +3785,7 @@
       </c>
       <c r="H66" s="4" t="inlineStr">
         <is>
-          <t>cod_mes=202605</t>
+          <t>cod_mes=202606</t>
         </is>
       </c>
       <c r="I66" s="4" t="inlineStr">
@@ -3795,7 +3795,7 @@
       </c>
       <c r="J66" s="4" t="inlineStr">
         <is>
-          <t>-1 mes</t>
+          <t>0 (anclaje 202606)</t>
         </is>
       </c>
     </row>
@@ -3835,7 +3835,7 @@
       </c>
       <c r="H67" s="7" t="inlineStr">
         <is>
-          <t>cod_mes=202605</t>
+          <t>cod_mes=202606</t>
         </is>
       </c>
       <c r="I67" s="7" t="inlineStr">
@@ -3845,7 +3845,7 @@
       </c>
       <c r="J67" s="7" t="inlineStr">
         <is>
-          <t>-1 mes</t>
+          <t>0 (anclaje 202606)</t>
         </is>
       </c>
     </row>
@@ -3885,7 +3885,7 @@
       </c>
       <c r="H68" s="4" t="inlineStr">
         <is>
-          <t>cod_mes=202605</t>
+          <t>cod_mes=202606</t>
         </is>
       </c>
       <c r="I68" s="4" t="inlineStr">
@@ -3895,7 +3895,7 @@
       </c>
       <c r="J68" s="4" t="inlineStr">
         <is>
-          <t>-1 mes</t>
+          <t>0 (anclaje 202606)</t>
         </is>
       </c>
     </row>
@@ -3935,7 +3935,7 @@
       </c>
       <c r="H69" s="7" t="inlineStr">
         <is>
-          <t>cod_mes 202605-202602</t>
+          <t>cod_mes 202606-202603</t>
         </is>
       </c>
       <c r="I69" s="7" t="inlineStr">
@@ -3945,7 +3945,7 @@
       </c>
       <c r="J69" s="7" t="inlineStr">
         <is>
-          <t>-1 a -4 meses</t>
+          <t>0 a -3 meses</t>
         </is>
       </c>
     </row>
@@ -3985,7 +3985,7 @@
       </c>
       <c r="H70" s="4" t="inlineStr">
         <is>
-          <t>cod_mes 202605-202512</t>
+          <t>cod_mes 202606-202601</t>
         </is>
       </c>
       <c r="I70" s="4" t="inlineStr">
@@ -3995,7 +3995,7 @@
       </c>
       <c r="J70" s="4" t="inlineStr">
         <is>
-          <t>-1 a -6 meses</t>
+          <t>0 a -5 meses</t>
         </is>
       </c>
     </row>
@@ -4035,7 +4035,7 @@
       </c>
       <c r="H71" s="7" t="inlineStr">
         <is>
-          <t>cod_mes 202605-202512</t>
+          <t>cod_mes 202606-202601</t>
         </is>
       </c>
       <c r="I71" s="7" t="inlineStr">
@@ -4045,7 +4045,7 @@
       </c>
       <c r="J71" s="7" t="inlineStr">
         <is>
-          <t>-1 a -6 meses</t>
+          <t>0 a -5 meses</t>
         </is>
       </c>
     </row>

</xml_diff>